<commit_message>
Case Blankenge with density added.
</commit_message>
<xml_diff>
--- a/Projects/Density/cases/RotatingIface/RotatingIface.xlsx
+++ b/Projects/Density/cases/RotatingIface/RotatingIface.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/GRWMODELS/python/mf6lab/Projects/Density/cases/RotatingIface/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39836110-CFF8-F148-9BB5-155877CBE837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F355861-59F0-DF4F-8AE4-2D6EE5448620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="-23740" windowWidth="30600" windowHeight="19860" tabRatio="751" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13624,7 +13624,7 @@
         <v>1</v>
       </c>
       <c r="B6">
-        <f>B5*tsmult</f>
+        <f t="shared" ref="B6:B18" si="0">B5*tsmult</f>
         <v>1.1000000000000001</v>
       </c>
       <c r="E6" s="11" t="s">
@@ -13640,7 +13640,7 @@
         <v>2</v>
       </c>
       <c r="B7">
-        <f>B6*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.2100000000000002</v>
       </c>
       <c r="F7">
@@ -13653,7 +13653,7 @@
         <v>3</v>
       </c>
       <c r="B8">
-        <f>B7*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.3310000000000004</v>
       </c>
       <c r="E8" s="11" t="s">
@@ -13668,7 +13668,7 @@
         <v>4</v>
       </c>
       <c r="B9">
-        <f>B8*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.4641000000000006</v>
       </c>
     </row>
@@ -13677,7 +13677,7 @@
         <v>5</v>
       </c>
       <c r="B10">
-        <f>B9*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.6105100000000008</v>
       </c>
     </row>
@@ -13686,7 +13686,7 @@
         <v>6</v>
       </c>
       <c r="B11">
-        <f>B10*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.7715610000000011</v>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
         <v>7</v>
       </c>
       <c r="B12">
-        <f>B11*tsmult</f>
+        <f t="shared" si="0"/>
         <v>1.9487171000000014</v>
       </c>
     </row>
@@ -13704,7 +13704,7 @@
         <v>8</v>
       </c>
       <c r="B13">
-        <f>B12*tsmult</f>
+        <f t="shared" si="0"/>
         <v>2.1435888100000016</v>
       </c>
     </row>
@@ -13713,7 +13713,7 @@
         <v>9</v>
       </c>
       <c r="B14">
-        <f>B13*tsmult</f>
+        <f t="shared" si="0"/>
         <v>2.3579476910000019</v>
       </c>
     </row>
@@ -13722,7 +13722,7 @@
         <v>10</v>
       </c>
       <c r="B15">
-        <f>B14*tsmult</f>
+        <f t="shared" si="0"/>
         <v>2.5937424601000023</v>
       </c>
     </row>
@@ -13731,7 +13731,7 @@
         <v>11</v>
       </c>
       <c r="B16">
-        <f>B15*tsmult</f>
+        <f t="shared" si="0"/>
         <v>2.8531167061100029</v>
       </c>
     </row>
@@ -13740,7 +13740,7 @@
         <v>12</v>
       </c>
       <c r="B17">
-        <f>B16*tsmult</f>
+        <f t="shared" si="0"/>
         <v>3.1384283767210035</v>
       </c>
     </row>
@@ -13749,7 +13749,7 @@
         <v>13</v>
       </c>
       <c r="B18">
-        <f>B17*tsmult</f>
+        <f t="shared" si="0"/>
         <v>3.4522712143931042</v>
       </c>
     </row>

</xml_diff>